<commit_message>
Atualizando banco de dados de contas tributárias
</commit_message>
<xml_diff>
--- a/banco_de_dados.xlsx
+++ b/banco_de_dados.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B30"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -427,6 +427,7 @@
           <t>3066</t>
         </is>
       </c>
+      <c r="C1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -439,6 +440,7 @@
           <t>2184</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -451,6 +453,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -463,6 +466,7 @@
           <t>2184</t>
         </is>
       </c>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -475,6 +479,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -487,6 +492,11 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -499,6 +509,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -511,6 +522,11 @@
           <t>3353</t>
         </is>
       </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -523,6 +539,7 @@
           <t>3353</t>
         </is>
       </c>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -535,6 +552,7 @@
           <t>3066</t>
         </is>
       </c>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -547,6 +565,7 @@
           <t>3353</t>
         </is>
       </c>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -559,6 +578,11 @@
           <t>3339</t>
         </is>
       </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -571,6 +595,11 @@
           <t>3066</t>
         </is>
       </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -583,6 +612,11 @@
           <t>3066</t>
         </is>
       </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -595,6 +629,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -607,6 +642,11 @@
           <t>2184</t>
         </is>
       </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -619,6 +659,7 @@
           <t>3066</t>
         </is>
       </c>
+      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -631,6 +672,7 @@
           <t>6102</t>
         </is>
       </c>
+      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -643,6 +685,7 @@
           <t>6102</t>
         </is>
       </c>
+      <c r="C19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -655,6 +698,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -667,6 +711,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -679,6 +724,11 @@
           <t>2184</t>
         </is>
       </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -691,6 +741,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -703,6 +754,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -715,6 +767,7 @@
           <t>6102</t>
         </is>
       </c>
+      <c r="C25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -727,6 +780,11 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -739,6 +797,7 @@
           <t>2184</t>
         </is>
       </c>
+      <c r="C27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -751,6 +810,11 @@
           <t>3066</t>
         </is>
       </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>325</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -763,6 +827,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -775,6 +840,7 @@
           <t>2135</t>
         </is>
       </c>
+      <c r="C30" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>